<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-20 22:20 UTC
</commit_message>
<xml_diff>
--- a/data/50001473 - MAPIMI.xlsx
+++ b/data/50001473 - MAPIMI.xlsx
@@ -4453,7 +4453,7 @@
       </c>
       <c r="C53" s="9"/>
       <c r="D53" s="8">
-        <v>46128.64908005787</v>
+        <v>46193.564339317134</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>172</v>
@@ -4498,9 +4498,11 @@
       <c r="B54" s="5">
         <v>46073.639872858796</v>
       </c>
-      <c r="C54" s="6"/>
+      <c r="C54" s="5">
+        <v>46193.56431931713</v>
+      </c>
       <c r="D54" s="5">
-        <v>46127.661168356484</v>
+        <v>46193.56432179398</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>202</v>
@@ -4624,9 +4626,11 @@
       <c r="B56" s="5">
         <v>46073.639869606486</v>
       </c>
-      <c r="C56" s="6"/>
+      <c r="C56" s="5">
+        <v>46193.56433421296</v>
+      </c>
       <c r="D56" s="5">
-        <v>46128.671001145834</v>
+        <v>46193.564335787036</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>207</v>
@@ -4752,7 +4756,7 @@
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46090.69359840278</v>
+        <v>46193.61410849537</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>213</v>
@@ -4797,9 +4801,11 @@
       <c r="B59" s="8">
         <v>46073.639870486106</v>
       </c>
-      <c r="C59" s="9"/>
+      <c r="C59" s="8">
+        <v>46193.61403773148</v>
+      </c>
       <c r="D59" s="8">
-        <v>46090.84579074074</v>
+        <v>46193.614040625005</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>216</v>
@@ -4860,9 +4866,11 @@
       <c r="B60" s="5">
         <v>46073.63987084491</v>
       </c>
-      <c r="C60" s="6"/>
+      <c r="C60" s="5">
+        <v>46193.61407924768</v>
+      </c>
       <c r="D60" s="5">
-        <v>46122.65691988426</v>
+        <v>46193.61408086805</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>219</v>
@@ -4921,9 +4929,11 @@
       <c r="B61" s="8">
         <v>46073.63987109954</v>
       </c>
-      <c r="C61" s="9"/>
+      <c r="C61" s="8">
+        <v>46193.6140899537</v>
+      </c>
       <c r="D61" s="8">
-        <v>46114.790324016205</v>
+        <v>46193.61409614583</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>223</v>
@@ -4984,9 +4994,11 @@
       <c r="B62" s="5">
         <v>46073.63987140046</v>
       </c>
-      <c r="C62" s="6"/>
+      <c r="C62" s="5">
+        <v>46193.61410039352</v>
+      </c>
       <c r="D62" s="5">
-        <v>46114.79032460648</v>
+        <v>46193.61410226852</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>226</v>
@@ -5049,7 +5061,7 @@
       </c>
       <c r="C63" s="9"/>
       <c r="D63" s="8">
-        <v>46090.84577681713</v>
+        <v>46193.614372870376</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>169</v>
@@ -5110,7 +5122,7 @@
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46090.84577170139</v>
+        <v>46193.564154085645</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>170</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-22 22:10 UTC
</commit_message>
<xml_diff>
--- a/data/50001473 - MAPIMI.xlsx
+++ b/data/50001473 - MAPIMI.xlsx
@@ -4215,7 +4215,7 @@
       </c>
       <c r="C49" s="9"/>
       <c r="D49" s="8">
-        <v>46191.881109062495</v>
+        <v>46195.913107650464</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>184</v>
@@ -4390,9 +4390,11 @@
       <c r="B52" s="5">
         <v>46073.63987233797</v>
       </c>
-      <c r="C52" s="6"/>
+      <c r="C52" s="5">
+        <v>46195.91309923611</v>
+      </c>
       <c r="D52" s="5">
-        <v>46191.88111327546</v>
+        <v>46195.9131012963</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>196</v>
@@ -4805,7 +4807,7 @@
         <v>46193.61403773148</v>
       </c>
       <c r="D59" s="8">
-        <v>46193.614040625005</v>
+        <v>46195.913108946756</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>216</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-23 14:01 UTC
</commit_message>
<xml_diff>
--- a/data/50001473 - MAPIMI.xlsx
+++ b/data/50001473 - MAPIMI.xlsx
@@ -5234,7 +5234,7 @@
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46195.567961782406</v>
+        <v>46196.58119877314</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>237</v>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46195.56842914352</v>
+        <v>46196.58146922453</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>244</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-25 14:10 UTC
</commit_message>
<xml_diff>
--- a/data/50001473 - MAPIMI.xlsx
+++ b/data/50001473 - MAPIMI.xlsx
@@ -3975,9 +3975,11 @@
       <c r="B45" s="8">
         <v>46090.67984755787</v>
       </c>
-      <c r="C45" s="9"/>
+      <c r="C45" s="8">
+        <v>46198.56751383102</v>
+      </c>
       <c r="D45" s="8">
-        <v>46195.56824368055</v>
+        <v>46198.567517812495</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>166</v>
@@ -5134,7 +5136,7 @@
         <v>46197.41887475694</v>
       </c>
       <c r="D64" s="5">
-        <v>46197.418877118056</v>
+        <v>46198.567522557874</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>170</v>

</xml_diff>